<commit_message>
fix: Add conditional use citizens/places_of_employment
The generic implementation in `competition.py` should either operate on
`citizens_per_class` or `places_of_employment` and the used data is
selected conditionally through the boolean flag `citizens` and assigned
into `citizens_or_places_of_employment`.

It turned out that towards the end of the script a plain instance of
`citizens_per_class` per class was used, without the conditional
selection based on the value of `citizens`.

This patch makes sure the conditional values in
`citizens_or_places_of_employment` are used here too.

The tests are updated accordingly.
</commit_message>
<xml_diff>
--- a/tests/vlaanderen/reference/resultaten/werk/concurrentie/arbeidsplaatsen/restdag/Ontpl_concproduct_Auto.xlsx
+++ b/tests/vlaanderen/reference/resultaten/werk/concurrentie/arbeidsplaatsen/restdag/Ontpl_concproduct_Auto.xlsx
@@ -385,16 +385,16 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>94.72654046762884</v>
+        <v>3.625896285842252</v>
       </c>
       <c r="C2">
-        <v>131.7440356678852</v>
+        <v>10.71602203997152</v>
       </c>
       <c r="D2">
-        <v>148.2345030934112</v>
+        <v>23.40544785685439</v>
       </c>
       <c r="E2">
-        <v>156.132524081533</v>
+        <v>37.53185675036851</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -402,16 +402,16 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>118.1753089179812</v>
+        <v>39.5525523725488</v>
       </c>
       <c r="C3">
-        <v>158.7526938108934</v>
+        <v>98.09109536282847</v>
       </c>
       <c r="D3">
-        <v>175.7004361084484</v>
+        <v>131.9546132406306</v>
       </c>
       <c r="E3">
-        <v>185.9889559210775</v>
+        <v>154.9907966008979</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -419,16 +419,16 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>103.2940631100031</v>
+        <v>3.922559358607711</v>
       </c>
       <c r="C4">
-        <v>147.8585557520053</v>
+        <v>10.56132541085753</v>
       </c>
       <c r="D4">
-        <v>168.3568331346805</v>
+        <v>19.17989238243195</v>
       </c>
       <c r="E4">
-        <v>178.8084080837329</v>
+        <v>26.29535412996072</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -436,16 +436,16 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>88.68178775961273</v>
+        <v>0</v>
       </c>
       <c r="C5">
-        <v>114.8114517912198</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>120.7087590389347</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>127.0603560451834</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -453,16 +453,16 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>76.64087752733985</v>
+        <v>25.72560923994624</v>
       </c>
       <c r="C6">
-        <v>99.0506165109433</v>
+        <v>42.25236088928351</v>
       </c>
       <c r="D6">
-        <v>106.4278641153051</v>
+        <v>41.67804468851107</v>
       </c>
       <c r="E6">
-        <v>110.9642725767895</v>
+        <v>35.9461728065656</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -470,16 +470,16 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>8.556061872758615</v>
+        <v>2.852020624252872</v>
       </c>
       <c r="C7">
-        <v>10.72557743548773</v>
+        <v>7.150384956991823</v>
       </c>
       <c r="D7">
-        <v>11.4513880430713</v>
+        <v>8.397684564918952</v>
       </c>
       <c r="E7">
-        <v>11.84143087829951</v>
+        <v>9.473144702639608</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -487,16 +487,16 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>283.1203258808434</v>
+        <v>0</v>
       </c>
       <c r="C8">
-        <v>441.9203503285401</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>537.287261301503</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>599.2709413296016</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -504,16 +504,16 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>115.7502609702506</v>
+        <v>207.9009541698676</v>
       </c>
       <c r="C9">
-        <v>143.5151943743134</v>
+        <v>411.1328998259315</v>
       </c>
       <c r="D9">
-        <v>151.612607300604</v>
+        <v>590.2587915295359</v>
       </c>
       <c r="E9">
-        <v>158.8511403311513</v>
+        <v>759.7228450620281</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -521,16 +521,16 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>50.03574183604502</v>
+        <v>0</v>
       </c>
       <c r="C10">
-        <v>61.53381390148514</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>66.20840949863424</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>67.5656795564007</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -538,16 +538,16 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>9.217870017468412</v>
+        <v>0</v>
       </c>
       <c r="C11">
-        <v>10.71019883711017</v>
+        <v>0</v>
       </c>
       <c r="D11">
-        <v>11.44193823086221</v>
+        <v>0</v>
       </c>
       <c r="E11">
-        <v>12.63740343921768</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -555,16 +555,16 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>24.77331179975072</v>
+        <v>304.2670859507844</v>
       </c>
       <c r="C12">
-        <v>29.25540472405986</v>
+        <v>390.5596530661992</v>
       </c>
       <c r="D12">
-        <v>30.37595654121452</v>
+        <v>343.2483089157241</v>
       </c>
       <c r="E12">
-        <v>30.46952081442694</v>
+        <v>265.6317199206451</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -572,16 +572,16 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>28.02784984031769</v>
+        <v>0</v>
       </c>
       <c r="C13">
-        <v>34.12210686605644</v>
+        <v>0</v>
       </c>
       <c r="D13">
-        <v>37.19404359333081</v>
+        <v>0</v>
       </c>
       <c r="E13">
-        <v>38.40936694258598</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>